<commit_message>
Add Azure DevOps pipeline and project dependencies
</commit_message>
<xml_diff>
--- a/datasets/hallucination_dataset_with_types.xlsx
+++ b/datasets/hallucination_dataset_with_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DeepEval\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF334DF6-92C1-4487-8B55-76A33E7BC7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F7224E-F718-4C4D-BCCB-982A235D8ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="factual_errors" sheetId="1" r:id="rId1"/>
@@ -532,6 +532,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>